<commit_message>
implement report type identification logic & implement architactuure
</commit_message>
<xml_diff>
--- a/export/a_r_25/v1.xlsx
+++ b/export/a_r_25/v1.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="נוכחות A" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="נוכחות A" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,8 +37,13 @@
       <b val="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="002C3E50"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -58,6 +63,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D5E8D4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EBF5FB"/>
       </patternFill>
     </fill>
   </fills>
@@ -87,7 +97,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -99,6 +109,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -466,7 +482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:K26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -585,8 +601,16 @@
           <t>2:00</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr"/>
-      <c r="K2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>0:00</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>0:00</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -629,9 +653,21 @@
           <t>7:20</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr"/>
-      <c r="J3" s="3" t="inlineStr"/>
-      <c r="K3" s="3" t="inlineStr"/>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>0:00</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>0:00</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>0:00</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -674,9 +710,21 @@
           <t>7:30</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr"/>
-      <c r="J4" s="2" t="inlineStr"/>
-      <c r="K4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>0:00</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>0:00</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>0:00</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -719,9 +767,21 @@
           <t>7:25</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr"/>
-      <c r="J5" s="3" t="inlineStr"/>
-      <c r="K5" s="3" t="inlineStr"/>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>0:00</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>0:00</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>0:00</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -764,9 +824,21 @@
           <t>7:35</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr"/>
-      <c r="J6" s="2" t="inlineStr"/>
-      <c r="K6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>0:00</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>0:00</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>0:00</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -814,8 +886,16 @@
           <t>2:00</t>
         </is>
       </c>
-      <c r="J7" s="3" t="inlineStr"/>
-      <c r="K7" s="3" t="inlineStr"/>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>0:00</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>0:00</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -858,9 +938,21 @@
           <t>7:30</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr"/>
-      <c r="J8" s="2" t="inlineStr"/>
-      <c r="K8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>0:00</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>0:00</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>0:00</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -903,9 +995,21 @@
           <t>7:05</t>
         </is>
       </c>
-      <c r="I9" s="3" t="inlineStr"/>
-      <c r="J9" s="3" t="inlineStr"/>
-      <c r="K9" s="3" t="inlineStr"/>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>0:00</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>0:00</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>0:00</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -948,9 +1052,21 @@
           <t>7:30</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr"/>
-      <c r="J10" s="2" t="inlineStr"/>
-      <c r="K10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>0:00</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>0:00</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>0:00</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -993,9 +1109,21 @@
           <t>7:20</t>
         </is>
       </c>
-      <c r="I11" s="3" t="inlineStr"/>
-      <c r="J11" s="3" t="inlineStr"/>
-      <c r="K11" s="3" t="inlineStr"/>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>0:00</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>0:00</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>0:00</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1043,8 +1171,16 @@
           <t>2:00</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr"/>
-      <c r="K12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>0:00</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>0:00</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -1087,9 +1223,21 @@
           <t>7:45</t>
         </is>
       </c>
-      <c r="I13" s="3" t="inlineStr"/>
-      <c r="J13" s="3" t="inlineStr"/>
-      <c r="K13" s="3" t="inlineStr"/>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>0:00</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>0:00</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>0:00</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1132,9 +1280,21 @@
           <t>7:40</t>
         </is>
       </c>
-      <c r="I14" s="2" t="inlineStr"/>
-      <c r="J14" s="2" t="inlineStr"/>
-      <c r="K14" s="2" t="inlineStr"/>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>0:00</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>0:00</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>0:00</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -1177,9 +1337,21 @@
           <t>7:45</t>
         </is>
       </c>
-      <c r="I15" s="3" t="inlineStr"/>
-      <c r="J15" s="3" t="inlineStr"/>
-      <c r="K15" s="3" t="inlineStr"/>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>0:00</t>
+        </is>
+      </c>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>0:00</t>
+        </is>
+      </c>
+      <c r="K15" s="3" t="inlineStr">
+        <is>
+          <t>0:00</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1222,9 +1394,21 @@
           <t>7:45</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr"/>
-      <c r="J16" s="2" t="inlineStr"/>
-      <c r="K16" s="2" t="inlineStr"/>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>0:00</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>0:00</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>0:00</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -1259,6 +1443,102 @@
       </c>
       <c r="K17" s="4" t="inlineStr"/>
     </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>ימים:</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>סה"כ שעות:</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>115:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>100% שעות:</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>109:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>125% שעות:</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>6:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>150% שעות:</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>0:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>שבת 150%:</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>0:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>בונוס:</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>נסיעות:</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Restructure into app/ package, add English docstrings, fix date/day reconstruction and ordering
</commit_message>
<xml_diff>
--- a/export/a_r_25/v1.xlsx
+++ b/export/a_r_25/v1.xlsx
@@ -482,7 +482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K26"/>
+  <dimension ref="A1:K25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -578,7 +578,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>16:50</t>
+          <t>15:50</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -588,17 +588,17 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>8:20</t>
+          <t>7:20</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>6:20</t>
+          <t>7:20</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>2:00</t>
+          <t>0:00</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -672,12 +672,12 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>05/02/2023</t>
+          <t>06/02/2023</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>ראשון</t>
+          <t>שני</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -687,12 +687,12 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>08:15</t>
+          <t>08:05</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>16:15</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -702,12 +702,12 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>7:30</t>
+          <t>7:25</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>7:30</t>
+          <t>7:25</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -729,12 +729,12 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>06/02/2023</t>
+          <t>07/02/2023</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>שני</t>
+          <t>שלישי</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -744,12 +744,12 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>08:05</t>
+          <t>08:15</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>16:15</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -759,12 +759,12 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>7:25</t>
+          <t>7:30</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>7:25</t>
+          <t>7:30</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
@@ -786,12 +786,12 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>07/02/2023</t>
+          <t>08/02/2023</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>שלישי</t>
+          <t>רביעי</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -801,12 +801,12 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>08:10</t>
+          <t>07:50</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>16:15</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -816,12 +816,12 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>7:35</t>
+          <t>7:40</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>7:35</t>
+          <t>7:40</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -843,12 +843,12 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>08/02/2023</t>
+          <t>09/02/2023</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>רביעי</t>
+          <t>חמישי</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -858,12 +858,12 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>07:50</t>
+          <t>08:45</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>16:45</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -873,17 +873,17 @@
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>8:40</t>
+          <t>7:30</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>6:40</t>
+          <t>7:30</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>2:00</t>
+          <t>0:00</t>
         </is>
       </c>
       <c r="J7" s="3" t="inlineStr">
@@ -900,12 +900,12 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>09/02/2023</t>
+          <t>12/02/2023</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>חמישי</t>
+          <t>ראשון</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -915,12 +915,12 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>08:15</t>
+          <t>09:15</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>16:15</t>
+          <t>16:50</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -930,12 +930,12 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>7:30</t>
+          <t>7:05</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>7:30</t>
+          <t>7:05</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -957,12 +957,12 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>12/02/2023</t>
+          <t>13/02/2023</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>ראשון</t>
+          <t>שני</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -972,12 +972,12 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>08:15</t>
+          <t>08:10</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>15:50</t>
+          <t>15:15</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -987,12 +987,12 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>7:05</t>
+          <t>6:35</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>7:05</t>
+          <t>6:35</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
@@ -1148,7 +1148,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -1158,17 +1158,17 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>8:30</t>
+          <t>7:30</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>6:30</t>
+          <t>7:30</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>2:00</t>
+          <t>0:00</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -1205,7 +1205,7 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
@@ -1215,12 +1215,12 @@
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>7:45</t>
+          <t>6:45</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>7:45</t>
+          <t>6:45</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr">
@@ -1354,147 +1354,102 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>21/02/2023</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>שלישי</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>סניף צפון</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>07:45</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>16:00</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>0:30</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>7:45</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>7:45</t>
-        </is>
-      </c>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>0:00</t>
-        </is>
-      </c>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>0:00</t>
-        </is>
-      </c>
-      <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t>0:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>סה"כ</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr"/>
-      <c r="C17" s="4" t="inlineStr"/>
-      <c r="D17" s="4" t="inlineStr"/>
-      <c r="E17" s="4" t="inlineStr"/>
-      <c r="F17" s="4" t="inlineStr"/>
-      <c r="G17" s="4" t="inlineStr">
-        <is>
-          <t>115:40</t>
-        </is>
-      </c>
-      <c r="H17" s="4" t="inlineStr">
-        <is>
-          <t>109:40</t>
-        </is>
-      </c>
-      <c r="I17" s="4" t="inlineStr">
-        <is>
-          <t>6:00</t>
-        </is>
-      </c>
-      <c r="J17" s="4" t="inlineStr">
-        <is>
-          <t>0:00</t>
-        </is>
-      </c>
-      <c r="K17" s="4" t="inlineStr"/>
+      <c r="B16" s="4" t="inlineStr"/>
+      <c r="C16" s="4" t="inlineStr"/>
+      <c r="D16" s="4" t="inlineStr"/>
+      <c r="E16" s="4" t="inlineStr"/>
+      <c r="F16" s="4" t="inlineStr"/>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>102:55</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>102:55</t>
+        </is>
+      </c>
+      <c r="I16" s="4" t="inlineStr">
+        <is>
+          <t>0:00</t>
+        </is>
+      </c>
+      <c r="J16" s="4" t="inlineStr">
+        <is>
+          <t>0:00</t>
+        </is>
+      </c>
+      <c r="K16" s="4" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>ימים:</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>ימים:</t>
+          <t>סה"כ שעות:</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>102:55</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>סה"כ שעות:</t>
+          <t>100% שעות:</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>115:40</t>
+          <t>102:55</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>100% שעות:</t>
+          <t>125% שעות:</t>
         </is>
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>109:40</t>
+          <t>0:00</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>125% שעות:</t>
+          <t>150% שעות:</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>6:00</t>
+          <t>0:00</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>150% שעות:</t>
+          <t>שבת 150%:</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
@@ -1506,34 +1461,22 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>שבת 150%:</t>
+          <t>בונוס:</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>0:00</t>
+          <t>0.00</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>בונוס:</t>
+          <t>נסיעות:</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
-        <is>
-          <t>0.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="5" t="inlineStr">
-        <is>
-          <t>נסיעות:</t>
-        </is>
-      </c>
-      <c r="B26" s="6" t="inlineStr">
         <is>
           <t>0.00</t>
         </is>

</xml_diff>